<commit_message>
fix: update equipment data with full excel import including 527 rods and 306 reels
</commit_message>
<xml_diff>
--- a/装备参数表.xlsx
+++ b/装备参数表.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1754" uniqueCount="961">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2058" uniqueCount="961">
   <si>
     <t>装备类型</t>
   </si>
@@ -9951,6 +9951,9 @@
       </c>
     </row>
     <row r="531" spans="1:3">
+      <c r="A531" t="s">
+        <v>5</v>
+      </c>
       <c r="B531" s="8" t="s">
         <v>656</v>
       </c>
@@ -9959,6 +9962,9 @@
       </c>
     </row>
     <row r="532" spans="1:3">
+      <c r="A532" t="s">
+        <v>5</v>
+      </c>
       <c r="B532" s="3" t="s">
         <v>657</v>
       </c>
@@ -9967,6 +9973,9 @@
       </c>
     </row>
     <row r="533" spans="1:3">
+      <c r="A533" t="s">
+        <v>5</v>
+      </c>
       <c r="B533" s="8" t="s">
         <v>658</v>
       </c>
@@ -9975,6 +9984,9 @@
       </c>
     </row>
     <row r="534" spans="1:3">
+      <c r="A534" t="s">
+        <v>5</v>
+      </c>
       <c r="B534" s="8" t="s">
         <v>659</v>
       </c>
@@ -9983,6 +9995,9 @@
       </c>
     </row>
     <row r="535" spans="1:3">
+      <c r="A535" t="s">
+        <v>5</v>
+      </c>
       <c r="B535" s="8" t="s">
         <v>660</v>
       </c>
@@ -9991,6 +10006,9 @@
       </c>
     </row>
     <row r="536" spans="1:3">
+      <c r="A536" t="s">
+        <v>5</v>
+      </c>
       <c r="B536" s="8" t="s">
         <v>661</v>
       </c>
@@ -9999,6 +10017,9 @@
       </c>
     </row>
     <row r="537" spans="1:3">
+      <c r="A537" t="s">
+        <v>5</v>
+      </c>
       <c r="B537" s="8" t="s">
         <v>662</v>
       </c>
@@ -10007,6 +10028,9 @@
       </c>
     </row>
     <row r="538" spans="1:3">
+      <c r="A538" t="s">
+        <v>5</v>
+      </c>
       <c r="B538" s="8" t="s">
         <v>663</v>
       </c>
@@ -10015,6 +10039,9 @@
       </c>
     </row>
     <row r="539" spans="1:3">
+      <c r="A539" t="s">
+        <v>5</v>
+      </c>
       <c r="B539" s="8" t="s">
         <v>664</v>
       </c>
@@ -10023,6 +10050,9 @@
       </c>
     </row>
     <row r="540" spans="1:3">
+      <c r="A540" t="s">
+        <v>5</v>
+      </c>
       <c r="B540" s="8" t="s">
         <v>666</v>
       </c>
@@ -10031,6 +10061,9 @@
       </c>
     </row>
     <row r="541" spans="1:3">
+      <c r="A541" t="s">
+        <v>5</v>
+      </c>
       <c r="B541" s="8" t="s">
         <v>667</v>
       </c>
@@ -10039,6 +10072,9 @@
       </c>
     </row>
     <row r="542" spans="1:3">
+      <c r="A542" t="s">
+        <v>5</v>
+      </c>
       <c r="B542" s="8" t="s">
         <v>668</v>
       </c>
@@ -10047,6 +10083,9 @@
       </c>
     </row>
     <row r="543" spans="1:3">
+      <c r="A543" t="s">
+        <v>5</v>
+      </c>
       <c r="B543" s="8" t="s">
         <v>669</v>
       </c>
@@ -10055,6 +10094,9 @@
       </c>
     </row>
     <row r="544" spans="1:3">
+      <c r="A544" t="s">
+        <v>5</v>
+      </c>
       <c r="B544" s="8" t="s">
         <v>670</v>
       </c>
@@ -10062,7 +10104,10 @@
         <v>31</v>
       </c>
     </row>
-    <row r="545" spans="2:3">
+    <row r="545" spans="1:3">
+      <c r="A545" t="s">
+        <v>5</v>
+      </c>
       <c r="B545" s="8" t="s">
         <v>671</v>
       </c>
@@ -10070,7 +10115,10 @@
         <v>37</v>
       </c>
     </row>
-    <row r="546" spans="2:3">
+    <row r="546" spans="1:3">
+      <c r="A546" t="s">
+        <v>5</v>
+      </c>
       <c r="B546" s="8" t="s">
         <v>672</v>
       </c>
@@ -10078,7 +10126,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="547" spans="2:3">
+    <row r="547" spans="1:3">
+      <c r="A547" t="s">
+        <v>5</v>
+      </c>
       <c r="B547" s="8" t="s">
         <v>673</v>
       </c>
@@ -10086,7 +10137,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="548" spans="2:3">
+    <row r="548" spans="1:3">
+      <c r="A548" t="s">
+        <v>5</v>
+      </c>
       <c r="B548" s="8" t="s">
         <v>674</v>
       </c>
@@ -10094,7 +10148,10 @@
         <v>28</v>
       </c>
     </row>
-    <row r="549" spans="2:3">
+    <row r="549" spans="1:3">
+      <c r="A549" t="s">
+        <v>5</v>
+      </c>
       <c r="B549" s="8" t="s">
         <v>675</v>
       </c>
@@ -10102,7 +10159,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="550" spans="2:3">
+    <row r="550" spans="1:3">
+      <c r="A550" t="s">
+        <v>5</v>
+      </c>
       <c r="B550" s="8" t="s">
         <v>676</v>
       </c>
@@ -10110,7 +10170,10 @@
         <v>41</v>
       </c>
     </row>
-    <row r="551" spans="2:3">
+    <row r="551" spans="1:3">
+      <c r="A551" t="s">
+        <v>5</v>
+      </c>
       <c r="B551" s="8" t="s">
         <v>677</v>
       </c>
@@ -10118,7 +10181,10 @@
         <v>80</v>
       </c>
     </row>
-    <row r="552" spans="2:3">
+    <row r="552" spans="1:3">
+      <c r="A552" t="s">
+        <v>5</v>
+      </c>
       <c r="B552" s="8" t="s">
         <v>678</v>
       </c>
@@ -10126,7 +10192,10 @@
         <v>67</v>
       </c>
     </row>
-    <row r="553" spans="2:3">
+    <row r="553" spans="1:3">
+      <c r="A553" t="s">
+        <v>5</v>
+      </c>
       <c r="B553" s="8" t="s">
         <v>679</v>
       </c>
@@ -10134,7 +10203,10 @@
         <v>72</v>
       </c>
     </row>
-    <row r="554" spans="2:3">
+    <row r="554" spans="1:3">
+      <c r="A554" t="s">
+        <v>5</v>
+      </c>
       <c r="B554" s="8" t="s">
         <v>680</v>
       </c>
@@ -10142,7 +10214,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="555" spans="2:3">
+    <row r="555" spans="1:3">
+      <c r="A555" t="s">
+        <v>5</v>
+      </c>
       <c r="B555" s="8" t="s">
         <v>681</v>
       </c>
@@ -10150,7 +10225,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="556" spans="2:3">
+    <row r="556" spans="1:3">
+      <c r="A556" t="s">
+        <v>5</v>
+      </c>
       <c r="B556" s="8" t="s">
         <v>682</v>
       </c>
@@ -10158,7 +10236,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="557" spans="2:3">
+    <row r="557" spans="1:3">
+      <c r="A557" t="s">
+        <v>5</v>
+      </c>
       <c r="B557" s="8" t="s">
         <v>683</v>
       </c>
@@ -10166,7 +10247,10 @@
         <v>14</v>
       </c>
     </row>
-    <row r="558" spans="2:3">
+    <row r="558" spans="1:3">
+      <c r="A558" t="s">
+        <v>5</v>
+      </c>
       <c r="B558" s="8" t="s">
         <v>684</v>
       </c>
@@ -10174,7 +10258,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="559" spans="2:3">
+    <row r="559" spans="1:3">
+      <c r="A559" t="s">
+        <v>5</v>
+      </c>
       <c r="B559" s="8" t="s">
         <v>685</v>
       </c>
@@ -10182,7 +10269,10 @@
         <v>17</v>
       </c>
     </row>
-    <row r="560" spans="2:3">
+    <row r="560" spans="1:3">
+      <c r="A560" t="s">
+        <v>5</v>
+      </c>
       <c r="B560" s="8" t="s">
         <v>686</v>
       </c>
@@ -10190,7 +10280,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="561" spans="2:3">
+    <row r="561" spans="1:3">
+      <c r="A561" t="s">
+        <v>5</v>
+      </c>
       <c r="B561" s="8" t="s">
         <v>687</v>
       </c>
@@ -10198,7 +10291,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="562" spans="2:3">
+    <row r="562" spans="1:3">
+      <c r="A562" t="s">
+        <v>5</v>
+      </c>
       <c r="B562" s="4" t="s">
         <v>688</v>
       </c>
@@ -10206,7 +10302,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="563" spans="2:3">
+    <row r="563" spans="1:3">
+      <c r="A563" t="s">
+        <v>5</v>
+      </c>
       <c r="B563" s="8" t="s">
         <v>689</v>
       </c>
@@ -10214,7 +10313,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="564" spans="2:3">
+    <row r="564" spans="1:3">
+      <c r="A564" t="s">
+        <v>5</v>
+      </c>
       <c r="B564" s="8" t="s">
         <v>690</v>
       </c>
@@ -10222,7 +10324,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="565" spans="2:3">
+    <row r="565" spans="1:3">
+      <c r="A565" t="s">
+        <v>5</v>
+      </c>
       <c r="B565" s="8" t="s">
         <v>691</v>
       </c>
@@ -10230,7 +10335,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="566" spans="2:3">
+    <row r="566" spans="1:3">
+      <c r="A566" t="s">
+        <v>5</v>
+      </c>
       <c r="B566" s="8" t="s">
         <v>692</v>
       </c>
@@ -10238,7 +10346,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="567" spans="2:3">
+    <row r="567" spans="1:3">
+      <c r="A567" t="s">
+        <v>5</v>
+      </c>
       <c r="B567" s="8" t="s">
         <v>693</v>
       </c>
@@ -10246,7 +10357,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="568" spans="2:3">
+    <row r="568" spans="1:3">
+      <c r="A568" t="s">
+        <v>5</v>
+      </c>
       <c r="B568" s="8" t="s">
         <v>694</v>
       </c>
@@ -10254,7 +10368,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="569" spans="2:3">
+    <row r="569" spans="1:3">
+      <c r="A569" t="s">
+        <v>5</v>
+      </c>
       <c r="B569" s="8" t="s">
         <v>695</v>
       </c>
@@ -10262,7 +10379,10 @@
         <v>17</v>
       </c>
     </row>
-    <row r="570" spans="2:3">
+    <row r="570" spans="1:3">
+      <c r="A570" t="s">
+        <v>5</v>
+      </c>
       <c r="B570" s="8" t="s">
         <v>696</v>
       </c>
@@ -10270,7 +10390,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="571" spans="2:3">
+    <row r="571" spans="1:3">
+      <c r="A571" t="s">
+        <v>5</v>
+      </c>
       <c r="B571" s="8" t="s">
         <v>697</v>
       </c>
@@ -10278,7 +10401,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="572" spans="2:3">
+    <row r="572" spans="1:3">
+      <c r="A572" t="s">
+        <v>5</v>
+      </c>
       <c r="B572" s="8" t="s">
         <v>698</v>
       </c>
@@ -10286,7 +10412,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="573" spans="2:3">
+    <row r="573" spans="1:3">
+      <c r="A573" t="s">
+        <v>5</v>
+      </c>
       <c r="B573" s="8" t="s">
         <v>699</v>
       </c>
@@ -10294,7 +10423,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="574" spans="2:3">
+    <row r="574" spans="1:3">
+      <c r="A574" t="s">
+        <v>5</v>
+      </c>
       <c r="B574" s="8" t="s">
         <v>700</v>
       </c>
@@ -10302,7 +10434,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="575" spans="2:3">
+    <row r="575" spans="1:3">
+      <c r="A575" t="s">
+        <v>5</v>
+      </c>
       <c r="B575" s="8" t="s">
         <v>701</v>
       </c>
@@ -10310,7 +10445,10 @@
         <v>45</v>
       </c>
     </row>
-    <row r="576" spans="2:3">
+    <row r="576" spans="1:3">
+      <c r="A576" t="s">
+        <v>5</v>
+      </c>
       <c r="B576" s="8" t="s">
         <v>702</v>
       </c>
@@ -10318,7 +10456,10 @@
         <v>45</v>
       </c>
     </row>
-    <row r="577" spans="2:3">
+    <row r="577" spans="1:3">
+      <c r="A577" t="s">
+        <v>5</v>
+      </c>
       <c r="B577" s="8" t="s">
         <v>703</v>
       </c>
@@ -10326,7 +10467,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="578" spans="2:3">
+    <row r="578" spans="1:3">
+      <c r="A578" t="s">
+        <v>5</v>
+      </c>
       <c r="B578" s="8" t="s">
         <v>704</v>
       </c>
@@ -10334,7 +10478,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="579" spans="2:3">
+    <row r="579" spans="1:3">
+      <c r="A579" t="s">
+        <v>5</v>
+      </c>
       <c r="B579" s="8" t="s">
         <v>705</v>
       </c>
@@ -10342,7 +10489,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="580" spans="2:3">
+    <row r="580" spans="1:3">
+      <c r="A580" t="s">
+        <v>5</v>
+      </c>
       <c r="B580" s="8" t="s">
         <v>706</v>
       </c>
@@ -10350,7 +10500,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="581" spans="2:3">
+    <row r="581" spans="1:3">
+      <c r="A581" t="s">
+        <v>5</v>
+      </c>
       <c r="B581" s="8" t="s">
         <v>707</v>
       </c>
@@ -10358,7 +10511,10 @@
         <v>72</v>
       </c>
     </row>
-    <row r="582" spans="2:3">
+    <row r="582" spans="1:3">
+      <c r="A582" t="s">
+        <v>5</v>
+      </c>
       <c r="B582" s="8" t="s">
         <v>708</v>
       </c>
@@ -10366,7 +10522,10 @@
         <v>49</v>
       </c>
     </row>
-    <row r="583" spans="2:3">
+    <row r="583" spans="1:3">
+      <c r="A583" t="s">
+        <v>5</v>
+      </c>
       <c r="B583" s="8" t="s">
         <v>709</v>
       </c>
@@ -10374,7 +10533,10 @@
         <v>9</v>
       </c>
     </row>
-    <row r="584" spans="2:3">
+    <row r="584" spans="1:3">
+      <c r="A584" t="s">
+        <v>5</v>
+      </c>
       <c r="B584" s="8" t="s">
         <v>710</v>
       </c>
@@ -10382,7 +10544,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="585" spans="2:3">
+    <row r="585" spans="1:3">
+      <c r="A585" t="s">
+        <v>5</v>
+      </c>
       <c r="B585" s="8" t="s">
         <v>711</v>
       </c>
@@ -10390,7 +10555,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="586" spans="2:3">
+    <row r="586" spans="1:3">
+      <c r="A586" t="s">
+        <v>5</v>
+      </c>
       <c r="B586" s="8" t="s">
         <v>712</v>
       </c>
@@ -10398,7 +10566,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="587" spans="2:3">
+    <row r="587" spans="1:3">
+      <c r="A587" t="s">
+        <v>5</v>
+      </c>
       <c r="B587" s="8" t="s">
         <v>713</v>
       </c>
@@ -10406,7 +10577,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="588" spans="2:3">
+    <row r="588" spans="1:3">
+      <c r="A588" t="s">
+        <v>5</v>
+      </c>
       <c r="B588" s="3" t="s">
         <v>714</v>
       </c>
@@ -10414,7 +10588,10 @@
         <v>5</v>
       </c>
     </row>
-    <row r="589" spans="2:3">
+    <row r="589" spans="1:3">
+      <c r="A589" t="s">
+        <v>5</v>
+      </c>
       <c r="B589" s="3" t="s">
         <v>715</v>
       </c>
@@ -10422,7 +10599,10 @@
         <v>5</v>
       </c>
     </row>
-    <row r="590" spans="2:3">
+    <row r="590" spans="1:3">
+      <c r="A590" t="s">
+        <v>5</v>
+      </c>
       <c r="B590" s="3" t="s">
         <v>716</v>
       </c>
@@ -10430,7 +10610,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="591" spans="2:3">
+    <row r="591" spans="1:3">
+      <c r="A591" t="s">
+        <v>5</v>
+      </c>
       <c r="B591" s="3" t="s">
         <v>717</v>
       </c>
@@ -10438,7 +10621,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="592" spans="2:3">
+    <row r="592" spans="1:3">
+      <c r="A592" t="s">
+        <v>5</v>
+      </c>
       <c r="B592" s="8" t="s">
         <v>718</v>
       </c>
@@ -10446,7 +10632,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="593" spans="2:3">
+    <row r="593" spans="1:3">
+      <c r="A593" t="s">
+        <v>5</v>
+      </c>
       <c r="B593" s="8" t="s">
         <v>719</v>
       </c>
@@ -10454,7 +10643,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="594" spans="2:3">
+    <row r="594" spans="1:3">
+      <c r="A594" t="s">
+        <v>5</v>
+      </c>
       <c r="B594" s="8" t="s">
         <v>720</v>
       </c>
@@ -10462,7 +10654,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="595" spans="2:3">
+    <row r="595" spans="1:3">
+      <c r="A595" t="s">
+        <v>5</v>
+      </c>
       <c r="B595" s="8" t="s">
         <v>721</v>
       </c>
@@ -10470,7 +10665,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="596" spans="2:3">
+    <row r="596" spans="1:3">
+      <c r="A596" t="s">
+        <v>5</v>
+      </c>
       <c r="B596" s="8" t="s">
         <v>722</v>
       </c>
@@ -10478,7 +10676,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="597" spans="2:3">
+    <row r="597" spans="1:3">
+      <c r="A597" t="s">
+        <v>5</v>
+      </c>
       <c r="B597" s="8" t="s">
         <v>723</v>
       </c>
@@ -10486,7 +10687,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="598" spans="2:3">
+    <row r="598" spans="1:3">
+      <c r="A598" t="s">
+        <v>5</v>
+      </c>
       <c r="B598" s="8" t="s">
         <v>724</v>
       </c>
@@ -10494,7 +10698,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="599" spans="2:3">
+    <row r="599" spans="1:3">
+      <c r="A599" t="s">
+        <v>5</v>
+      </c>
       <c r="B599" s="8" t="s">
         <v>725</v>
       </c>
@@ -10502,7 +10709,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="600" spans="2:3">
+    <row r="600" spans="1:3">
+      <c r="A600" t="s">
+        <v>5</v>
+      </c>
       <c r="B600" s="8" t="s">
         <v>726</v>
       </c>
@@ -10510,7 +10720,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="601" spans="2:3">
+    <row r="601" spans="1:3">
+      <c r="A601" t="s">
+        <v>5</v>
+      </c>
       <c r="B601" s="8" t="s">
         <v>727</v>
       </c>
@@ -10518,7 +10731,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="602" spans="2:3">
+    <row r="602" spans="1:3">
+      <c r="A602" t="s">
+        <v>5</v>
+      </c>
       <c r="B602" s="8" t="s">
         <v>728</v>
       </c>
@@ -10526,7 +10742,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="603" spans="2:3">
+    <row r="603" spans="1:3">
+      <c r="A603" t="s">
+        <v>5</v>
+      </c>
       <c r="B603" s="8" t="s">
         <v>729</v>
       </c>
@@ -10534,7 +10753,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="604" spans="2:3">
+    <row r="604" spans="1:3">
+      <c r="A604" t="s">
+        <v>5</v>
+      </c>
       <c r="B604" s="8" t="s">
         <v>730</v>
       </c>
@@ -10542,7 +10764,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="605" spans="2:3">
+    <row r="605" spans="1:3">
+      <c r="A605" t="s">
+        <v>5</v>
+      </c>
       <c r="B605" s="8" t="s">
         <v>731</v>
       </c>
@@ -10550,7 +10775,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="606" spans="2:3">
+    <row r="606" spans="1:3">
+      <c r="A606" t="s">
+        <v>5</v>
+      </c>
       <c r="B606" s="8" t="s">
         <v>732</v>
       </c>
@@ -10558,7 +10786,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="607" spans="2:3">
+    <row r="607" spans="1:3">
+      <c r="A607" t="s">
+        <v>5</v>
+      </c>
       <c r="B607" s="8" t="s">
         <v>733</v>
       </c>
@@ -10566,7 +10797,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="608" spans="2:3">
+    <row r="608" spans="1:3">
+      <c r="A608" t="s">
+        <v>5</v>
+      </c>
       <c r="B608" s="8" t="s">
         <v>734</v>
       </c>
@@ -10574,7 +10808,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="609" spans="2:3">
+    <row r="609" spans="1:3">
+      <c r="A609" t="s">
+        <v>5</v>
+      </c>
       <c r="B609" s="8" t="s">
         <v>735</v>
       </c>
@@ -10582,7 +10819,10 @@
         <v>34</v>
       </c>
     </row>
-    <row r="610" spans="2:3">
+    <row r="610" spans="1:3">
+      <c r="A610" t="s">
+        <v>5</v>
+      </c>
       <c r="B610" s="8" t="s">
         <v>736</v>
       </c>
@@ -10590,7 +10830,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="611" spans="2:3">
+    <row r="611" spans="1:3">
+      <c r="A611" t="s">
+        <v>5</v>
+      </c>
       <c r="B611" s="8" t="s">
         <v>737</v>
       </c>
@@ -10598,7 +10841,10 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="612" spans="2:3">
+    <row r="612" spans="1:3">
+      <c r="A612" t="s">
+        <v>5</v>
+      </c>
       <c r="B612" s="8" t="s">
         <v>738</v>
       </c>
@@ -10606,7 +10852,10 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="613" spans="2:3">
+    <row r="613" spans="1:3">
+      <c r="A613" t="s">
+        <v>5</v>
+      </c>
       <c r="B613" s="8" t="s">
         <v>739</v>
       </c>
@@ -10614,7 +10863,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="614" spans="2:3">
+    <row r="614" spans="1:3">
+      <c r="A614" t="s">
+        <v>5</v>
+      </c>
       <c r="B614" s="8" t="s">
         <v>740</v>
       </c>
@@ -10622,7 +10874,10 @@
         <v>18</v>
       </c>
     </row>
-    <row r="615" spans="2:3">
+    <row r="615" spans="1:3">
+      <c r="A615" t="s">
+        <v>5</v>
+      </c>
       <c r="B615" s="8" t="s">
         <v>741</v>
       </c>
@@ -10630,7 +10885,10 @@
         <v>22</v>
       </c>
     </row>
-    <row r="616" spans="2:3">
+    <row r="616" spans="1:3">
+      <c r="A616" t="s">
+        <v>5</v>
+      </c>
       <c r="B616" s="8" t="s">
         <v>742</v>
       </c>
@@ -10638,7 +10896,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="617" spans="2:3">
+    <row r="617" spans="1:3">
+      <c r="A617" t="s">
+        <v>5</v>
+      </c>
       <c r="B617" s="8" t="s">
         <v>743</v>
       </c>
@@ -10646,7 +10907,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="618" spans="2:3">
+    <row r="618" spans="1:3">
+      <c r="A618" t="s">
+        <v>5</v>
+      </c>
       <c r="B618" s="8" t="s">
         <v>744</v>
       </c>
@@ -10654,7 +10918,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="619" spans="2:3">
+    <row r="619" spans="1:3">
+      <c r="A619" t="s">
+        <v>5</v>
+      </c>
       <c r="B619" s="8" t="s">
         <v>745</v>
       </c>
@@ -10662,7 +10929,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="620" spans="2:3">
+    <row r="620" spans="1:3">
+      <c r="A620" t="s">
+        <v>5</v>
+      </c>
       <c r="B620" s="8" t="s">
         <v>746</v>
       </c>
@@ -10670,7 +10940,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="621" spans="2:3">
+    <row r="621" spans="1:3">
+      <c r="A621" t="s">
+        <v>5</v>
+      </c>
       <c r="B621" s="8" t="s">
         <v>747</v>
       </c>
@@ -10678,7 +10951,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="622" spans="2:3">
+    <row r="622" spans="1:3">
+      <c r="A622" t="s">
+        <v>5</v>
+      </c>
       <c r="B622" s="8" t="s">
         <v>748</v>
       </c>
@@ -10686,7 +10962,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="623" spans="2:3">
+    <row r="623" spans="1:3">
+      <c r="A623" t="s">
+        <v>5</v>
+      </c>
       <c r="B623" s="8" t="s">
         <v>749</v>
       </c>
@@ -10694,7 +10973,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="624" spans="2:3">
+    <row r="624" spans="1:3">
+      <c r="A624" t="s">
+        <v>5</v>
+      </c>
       <c r="B624" s="8" t="s">
         <v>750</v>
       </c>
@@ -10702,7 +10984,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="625" spans="2:3">
+    <row r="625" spans="1:3">
+      <c r="A625" t="s">
+        <v>5</v>
+      </c>
       <c r="B625" s="8" t="s">
         <v>751</v>
       </c>
@@ -10710,7 +10995,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="626" spans="2:3">
+    <row r="626" spans="1:3">
+      <c r="A626" t="s">
+        <v>5</v>
+      </c>
       <c r="B626" s="8" t="s">
         <v>752</v>
       </c>
@@ -10718,7 +11006,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="627" spans="2:3">
+    <row r="627" spans="1:3">
+      <c r="A627" t="s">
+        <v>5</v>
+      </c>
       <c r="B627" s="8" t="s">
         <v>753</v>
       </c>
@@ -10726,7 +11017,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="628" spans="2:3">
+    <row r="628" spans="1:3">
+      <c r="A628" t="s">
+        <v>5</v>
+      </c>
       <c r="B628" s="8" t="s">
         <v>754</v>
       </c>
@@ -10734,7 +11028,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="629" spans="2:3">
+    <row r="629" spans="1:3">
+      <c r="A629" t="s">
+        <v>5</v>
+      </c>
       <c r="B629" s="8" t="s">
         <v>755</v>
       </c>
@@ -10742,7 +11039,10 @@
         <v>25</v>
       </c>
     </row>
-    <row r="630" spans="2:3">
+    <row r="630" spans="1:3">
+      <c r="A630" t="s">
+        <v>5</v>
+      </c>
       <c r="B630" s="8" t="s">
         <v>756</v>
       </c>
@@ -10750,7 +11050,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="631" spans="2:3">
+    <row r="631" spans="1:3">
+      <c r="A631" t="s">
+        <v>5</v>
+      </c>
       <c r="B631" s="8" t="s">
         <v>757</v>
       </c>
@@ -10758,7 +11061,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="632" spans="2:3">
+    <row r="632" spans="1:3">
+      <c r="A632" t="s">
+        <v>5</v>
+      </c>
       <c r="B632" s="8" t="s">
         <v>758</v>
       </c>
@@ -10766,7 +11072,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="633" spans="2:3">
+    <row r="633" spans="1:3">
+      <c r="A633" t="s">
+        <v>5</v>
+      </c>
       <c r="B633" s="8" t="s">
         <v>759</v>
       </c>
@@ -10774,7 +11083,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="634" spans="2:3">
+    <row r="634" spans="1:3">
+      <c r="A634" t="s">
+        <v>5</v>
+      </c>
       <c r="B634" s="8" t="s">
         <v>760</v>
       </c>
@@ -10782,7 +11094,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="635" spans="2:3">
+    <row r="635" spans="1:3">
+      <c r="A635" t="s">
+        <v>5</v>
+      </c>
       <c r="B635" s="8" t="s">
         <v>761</v>
       </c>
@@ -10790,7 +11105,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="636" spans="2:3">
+    <row r="636" spans="1:3">
+      <c r="A636" t="s">
+        <v>5</v>
+      </c>
       <c r="B636" s="8" t="s">
         <v>762</v>
       </c>
@@ -10798,7 +11116,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="637" spans="2:3">
+    <row r="637" spans="1:3">
+      <c r="A637" t="s">
+        <v>5</v>
+      </c>
       <c r="B637" s="8" t="s">
         <v>763</v>
       </c>
@@ -10806,7 +11127,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="638" spans="2:3">
+    <row r="638" spans="1:3">
+      <c r="A638" t="s">
+        <v>5</v>
+      </c>
       <c r="B638" s="8" t="s">
         <v>764</v>
       </c>
@@ -10814,13 +11138,19 @@
         <v>665</v>
       </c>
     </row>
-    <row r="639" spans="2:3">
+    <row r="639" spans="1:3">
+      <c r="A639" t="s">
+        <v>5</v>
+      </c>
       <c r="B639" s="8" t="s">
         <v>765</v>
       </c>
       <c r="C639" s="8"/>
     </row>
-    <row r="640" spans="2:3">
+    <row r="640" spans="1:3">
+      <c r="A640" t="s">
+        <v>5</v>
+      </c>
       <c r="B640" s="8" t="s">
         <v>766</v>
       </c>
@@ -10828,7 +11158,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="641" spans="2:3">
+    <row r="641" spans="1:3">
+      <c r="A641" t="s">
+        <v>5</v>
+      </c>
       <c r="B641" s="8" t="s">
         <v>767</v>
       </c>
@@ -10836,7 +11169,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="642" spans="2:3">
+    <row r="642" spans="1:3">
+      <c r="A642" t="s">
+        <v>5</v>
+      </c>
       <c r="B642" s="8" t="s">
         <v>768</v>
       </c>
@@ -10844,7 +11180,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="643" spans="2:3">
+    <row r="643" spans="1:3">
+      <c r="A643" t="s">
+        <v>5</v>
+      </c>
       <c r="B643" s="8" t="s">
         <v>769</v>
       </c>
@@ -10852,7 +11191,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="644" spans="2:3">
+    <row r="644" spans="1:3">
+      <c r="A644" t="s">
+        <v>5</v>
+      </c>
       <c r="B644" s="8" t="s">
         <v>770</v>
       </c>
@@ -10860,7 +11202,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="645" spans="2:3">
+    <row r="645" spans="1:3">
+      <c r="A645" t="s">
+        <v>5</v>
+      </c>
       <c r="B645" s="8" t="s">
         <v>771</v>
       </c>
@@ -10868,7 +11213,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="646" spans="2:3">
+    <row r="646" spans="1:3">
+      <c r="A646" t="s">
+        <v>5</v>
+      </c>
       <c r="B646" s="8" t="s">
         <v>772</v>
       </c>
@@ -10876,7 +11224,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="647" spans="2:3">
+    <row r="647" spans="1:3">
+      <c r="A647" t="s">
+        <v>5</v>
+      </c>
       <c r="B647" s="8" t="s">
         <v>773</v>
       </c>
@@ -10884,7 +11235,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="648" spans="2:3">
+    <row r="648" spans="1:3">
+      <c r="A648" t="s">
+        <v>5</v>
+      </c>
       <c r="B648" s="8" t="s">
         <v>774</v>
       </c>
@@ -10892,7 +11246,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="649" spans="2:3">
+    <row r="649" spans="1:3">
+      <c r="A649" t="s">
+        <v>5</v>
+      </c>
       <c r="B649" s="8" t="s">
         <v>775</v>
       </c>
@@ -10900,7 +11257,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="650" spans="2:3">
+    <row r="650" spans="1:3">
+      <c r="A650" t="s">
+        <v>5</v>
+      </c>
       <c r="B650" s="8" t="s">
         <v>776</v>
       </c>
@@ -10908,7 +11268,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="651" spans="2:3">
+    <row r="651" spans="1:3">
+      <c r="A651" t="s">
+        <v>5</v>
+      </c>
       <c r="B651" s="8" t="s">
         <v>777</v>
       </c>
@@ -10916,7 +11279,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="652" spans="2:3">
+    <row r="652" spans="1:3">
+      <c r="A652" t="s">
+        <v>5</v>
+      </c>
       <c r="B652" s="3" t="s">
         <v>778</v>
       </c>
@@ -10924,7 +11290,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="653" spans="2:3">
+    <row r="653" spans="1:3">
+      <c r="A653" t="s">
+        <v>5</v>
+      </c>
       <c r="B653" s="8" t="s">
         <v>779</v>
       </c>
@@ -10932,7 +11301,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="654" spans="2:3">
+    <row r="654" spans="1:3">
+      <c r="A654" t="s">
+        <v>5</v>
+      </c>
       <c r="B654" s="8" t="s">
         <v>780</v>
       </c>
@@ -10940,7 +11312,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="655" spans="2:3">
+    <row r="655" spans="1:3">
+      <c r="A655" t="s">
+        <v>5</v>
+      </c>
       <c r="B655" s="8" t="s">
         <v>781</v>
       </c>
@@ -10948,7 +11323,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="656" spans="2:3">
+    <row r="656" spans="1:3">
+      <c r="A656" t="s">
+        <v>5</v>
+      </c>
       <c r="B656" s="8" t="s">
         <v>782</v>
       </c>
@@ -10956,7 +11334,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="657" spans="2:3">
+    <row r="657" spans="1:3">
+      <c r="A657" t="s">
+        <v>5</v>
+      </c>
       <c r="B657" s="3" t="s">
         <v>783</v>
       </c>
@@ -10964,7 +11345,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="658" spans="2:3">
+    <row r="658" spans="1:3">
+      <c r="A658" t="s">
+        <v>5</v>
+      </c>
       <c r="B658" s="8" t="s">
         <v>784</v>
       </c>
@@ -10972,7 +11356,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="659" spans="2:3">
+    <row r="659" spans="1:3">
+      <c r="A659" t="s">
+        <v>5</v>
+      </c>
       <c r="B659" s="8" t="s">
         <v>785</v>
       </c>
@@ -10980,7 +11367,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="660" spans="2:3">
+    <row r="660" spans="1:3">
+      <c r="A660" t="s">
+        <v>5</v>
+      </c>
       <c r="B660" s="8" t="s">
         <v>786</v>
       </c>
@@ -10988,7 +11378,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="661" spans="2:3">
+    <row r="661" spans="1:3">
+      <c r="A661" t="s">
+        <v>5</v>
+      </c>
       <c r="B661" s="8" t="s">
         <v>787</v>
       </c>
@@ -10996,7 +11389,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="662" spans="2:3">
+    <row r="662" spans="1:3">
+      <c r="A662" t="s">
+        <v>5</v>
+      </c>
       <c r="B662" s="8" t="s">
         <v>788</v>
       </c>
@@ -11004,7 +11400,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="663" spans="2:3">
+    <row r="663" spans="1:3">
+      <c r="A663" t="s">
+        <v>5</v>
+      </c>
       <c r="B663" s="8" t="s">
         <v>789</v>
       </c>
@@ -11012,7 +11411,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="664" spans="2:3">
+    <row r="664" spans="1:3">
+      <c r="A664" t="s">
+        <v>5</v>
+      </c>
       <c r="B664" s="8" t="s">
         <v>790</v>
       </c>
@@ -11020,7 +11422,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="665" spans="2:3">
+    <row r="665" spans="1:3">
+      <c r="A665" t="s">
+        <v>5</v>
+      </c>
       <c r="B665" s="8" t="s">
         <v>791</v>
       </c>
@@ -11028,7 +11433,10 @@
         <v>11</v>
       </c>
     </row>
-    <row r="666" spans="2:3">
+    <row r="666" spans="1:3">
+      <c r="A666" t="s">
+        <v>5</v>
+      </c>
       <c r="B666" s="3" t="s">
         <v>792</v>
       </c>
@@ -11036,7 +11444,10 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="667" spans="2:3">
+    <row r="667" spans="1:3">
+      <c r="A667" t="s">
+        <v>5</v>
+      </c>
       <c r="B667" s="8" t="s">
         <v>793</v>
       </c>
@@ -11044,7 +11455,10 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="668" spans="2:3">
+    <row r="668" spans="1:3">
+      <c r="A668" t="s">
+        <v>5</v>
+      </c>
       <c r="B668" s="8" t="s">
         <v>794</v>
       </c>
@@ -11052,7 +11466,10 @@
         <v>4</v>
       </c>
     </row>
-    <row r="669" spans="2:3">
+    <row r="669" spans="1:3">
+      <c r="A669" t="s">
+        <v>5</v>
+      </c>
       <c r="B669" s="8" t="s">
         <v>795</v>
       </c>
@@ -11060,7 +11477,10 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="670" spans="2:3">
+    <row r="670" spans="1:3">
+      <c r="A670" t="s">
+        <v>5</v>
+      </c>
       <c r="B670" s="8" t="s">
         <v>796</v>
       </c>
@@ -11068,7 +11488,10 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="671" spans="2:3">
+    <row r="671" spans="1:3">
+      <c r="A671" t="s">
+        <v>5</v>
+      </c>
       <c r="B671" s="8" t="s">
         <v>797</v>
       </c>
@@ -11076,7 +11499,10 @@
         <v>4</v>
       </c>
     </row>
-    <row r="672" spans="2:3">
+    <row r="672" spans="1:3">
+      <c r="A672" t="s">
+        <v>5</v>
+      </c>
       <c r="B672" s="8" t="s">
         <v>798</v>
       </c>
@@ -11084,7 +11510,10 @@
         <v>5</v>
       </c>
     </row>
-    <row r="673" spans="2:3">
+    <row r="673" spans="1:3">
+      <c r="A673" t="s">
+        <v>5</v>
+      </c>
       <c r="B673" s="8" t="s">
         <v>799</v>
       </c>
@@ -11092,7 +11521,10 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="674" spans="2:3">
+    <row r="674" spans="1:3">
+      <c r="A674" t="s">
+        <v>5</v>
+      </c>
       <c r="B674" s="8" t="s">
         <v>800</v>
       </c>
@@ -11100,7 +11532,10 @@
         <v>2</v>
       </c>
     </row>
-    <row r="675" spans="2:3">
+    <row r="675" spans="1:3">
+      <c r="A675" t="s">
+        <v>5</v>
+      </c>
       <c r="B675" s="8" t="s">
         <v>801</v>
       </c>
@@ -11108,7 +11543,10 @@
         <v>2</v>
       </c>
     </row>
-    <row r="676" spans="2:3">
+    <row r="676" spans="1:3">
+      <c r="A676" t="s">
+        <v>5</v>
+      </c>
       <c r="B676" s="8" t="s">
         <v>802</v>
       </c>
@@ -11116,7 +11554,10 @@
         <v>2</v>
       </c>
     </row>
-    <row r="677" spans="2:3">
+    <row r="677" spans="1:3">
+      <c r="A677" t="s">
+        <v>5</v>
+      </c>
       <c r="B677" s="8" t="s">
         <v>803</v>
       </c>
@@ -11124,7 +11565,10 @@
         <v>5</v>
       </c>
     </row>
-    <row r="678" spans="2:3">
+    <row r="678" spans="1:3">
+      <c r="A678" t="s">
+        <v>5</v>
+      </c>
       <c r="B678" s="8" t="s">
         <v>804</v>
       </c>
@@ -11132,7 +11576,10 @@
         <v>5</v>
       </c>
     </row>
-    <row r="679" spans="2:3">
+    <row r="679" spans="1:3">
+      <c r="A679" t="s">
+        <v>5</v>
+      </c>
       <c r="B679" s="8" t="s">
         <v>805</v>
       </c>
@@ -11140,7 +11587,10 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="680" spans="2:3">
+    <row r="680" spans="1:3">
+      <c r="A680" t="s">
+        <v>5</v>
+      </c>
       <c r="B680" s="8" t="s">
         <v>806</v>
       </c>
@@ -11148,7 +11598,10 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="681" spans="2:3">
+    <row r="681" spans="1:3">
+      <c r="A681" t="s">
+        <v>5</v>
+      </c>
       <c r="B681" s="8" t="s">
         <v>807</v>
       </c>
@@ -11156,7 +11609,10 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="682" spans="2:3">
+    <row r="682" spans="1:3">
+      <c r="A682" t="s">
+        <v>5</v>
+      </c>
       <c r="B682" s="8" t="s">
         <v>808</v>
       </c>
@@ -11164,7 +11620,10 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="683" spans="2:3">
+    <row r="683" spans="1:3">
+      <c r="A683" t="s">
+        <v>5</v>
+      </c>
       <c r="B683" s="8" t="s">
         <v>809</v>
       </c>
@@ -11172,7 +11631,10 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="684" spans="2:3">
+    <row r="684" spans="1:3">
+      <c r="A684" t="s">
+        <v>5</v>
+      </c>
       <c r="B684" s="8" t="s">
         <v>810</v>
       </c>
@@ -11180,7 +11642,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="685" spans="2:3">
+    <row r="685" spans="1:3">
+      <c r="A685" t="s">
+        <v>5</v>
+      </c>
       <c r="B685" s="8" t="s">
         <v>811</v>
       </c>
@@ -11188,7 +11653,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="686" spans="2:3">
+    <row r="686" spans="1:3">
+      <c r="A686" t="s">
+        <v>5</v>
+      </c>
       <c r="B686" s="8" t="s">
         <v>812</v>
       </c>
@@ -11196,7 +11664,10 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="687" spans="2:3">
+    <row r="687" spans="1:3">
+      <c r="A687" t="s">
+        <v>5</v>
+      </c>
       <c r="B687" s="8" t="s">
         <v>813</v>
       </c>
@@ -11204,7 +11675,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="688" spans="2:3">
+    <row r="688" spans="1:3">
+      <c r="A688" t="s">
+        <v>5</v>
+      </c>
       <c r="B688" s="8" t="s">
         <v>814</v>
       </c>
@@ -11212,7 +11686,10 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="689" spans="2:3">
+    <row r="689" spans="1:3">
+      <c r="A689" t="s">
+        <v>5</v>
+      </c>
       <c r="B689" s="8" t="s">
         <v>815</v>
       </c>
@@ -11220,7 +11697,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="690" spans="2:3">
+    <row r="690" spans="1:3">
+      <c r="A690" t="s">
+        <v>5</v>
+      </c>
       <c r="B690" s="3" t="s">
         <v>816</v>
       </c>
@@ -11228,7 +11708,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="691" spans="2:3">
+    <row r="691" spans="1:3">
+      <c r="A691" t="s">
+        <v>5</v>
+      </c>
       <c r="B691" s="8" t="s">
         <v>817</v>
       </c>
@@ -11236,7 +11719,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="692" spans="2:3">
+    <row r="692" spans="1:3">
+      <c r="A692" t="s">
+        <v>5</v>
+      </c>
       <c r="B692" s="8" t="s">
         <v>818</v>
       </c>
@@ -11244,7 +11730,10 @@
         <v>38</v>
       </c>
     </row>
-    <row r="693" spans="2:3">
+    <row r="693" spans="1:3">
+      <c r="A693" t="s">
+        <v>5</v>
+      </c>
       <c r="B693" s="3" t="s">
         <v>819</v>
       </c>
@@ -11252,7 +11741,10 @@
         <v>28</v>
       </c>
     </row>
-    <row r="694" spans="2:3">
+    <row r="694" spans="1:3">
+      <c r="A694" t="s">
+        <v>5</v>
+      </c>
       <c r="B694" s="3" t="s">
         <v>820</v>
       </c>
@@ -11260,7 +11752,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="695" spans="2:3">
+    <row r="695" spans="1:3">
+      <c r="A695" t="s">
+        <v>5</v>
+      </c>
       <c r="B695" s="8" t="s">
         <v>821</v>
       </c>
@@ -11268,7 +11763,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="696" spans="2:3">
+    <row r="696" spans="1:3">
+      <c r="A696" t="s">
+        <v>5</v>
+      </c>
       <c r="B696" s="8" t="s">
         <v>822</v>
       </c>
@@ -11276,7 +11774,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="697" spans="2:3">
+    <row r="697" spans="1:3">
+      <c r="A697" t="s">
+        <v>5</v>
+      </c>
       <c r="B697" s="8" t="s">
         <v>823</v>
       </c>
@@ -11284,7 +11785,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="698" spans="2:3">
+    <row r="698" spans="1:3">
+      <c r="A698" t="s">
+        <v>5</v>
+      </c>
       <c r="B698" s="8" t="s">
         <v>824</v>
       </c>
@@ -11292,7 +11796,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="699" spans="2:3">
+    <row r="699" spans="1:3">
+      <c r="A699" t="s">
+        <v>5</v>
+      </c>
       <c r="B699" s="8" t="s">
         <v>825</v>
       </c>
@@ -11300,7 +11807,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="700" spans="2:3">
+    <row r="700" spans="1:3">
+      <c r="A700" t="s">
+        <v>5</v>
+      </c>
       <c r="B700" s="3" t="s">
         <v>826</v>
       </c>
@@ -11308,7 +11818,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="701" spans="2:3">
+    <row r="701" spans="1:3">
+      <c r="A701" t="s">
+        <v>5</v>
+      </c>
       <c r="B701" s="8" t="s">
         <v>827</v>
       </c>
@@ -11316,7 +11829,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="702" spans="2:3">
+    <row r="702" spans="1:3">
+      <c r="A702" t="s">
+        <v>5</v>
+      </c>
       <c r="B702" s="8" t="s">
         <v>828</v>
       </c>
@@ -11324,7 +11840,10 @@
         <v>21</v>
       </c>
     </row>
-    <row r="703" spans="2:3">
+    <row r="703" spans="1:3">
+      <c r="A703" t="s">
+        <v>5</v>
+      </c>
       <c r="B703" s="8" t="s">
         <v>829</v>
       </c>
@@ -11332,7 +11851,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="704" spans="2:3">
+    <row r="704" spans="1:3">
+      <c r="A704" t="s">
+        <v>5</v>
+      </c>
       <c r="B704" s="8" t="s">
         <v>830</v>
       </c>
@@ -11340,7 +11862,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="705" spans="2:3">
+    <row r="705" spans="1:3">
+      <c r="A705" t="s">
+        <v>5</v>
+      </c>
       <c r="B705" s="8" t="s">
         <v>831</v>
       </c>
@@ -11348,7 +11873,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="706" spans="2:3">
+    <row r="706" spans="1:3">
+      <c r="A706" t="s">
+        <v>5</v>
+      </c>
       <c r="B706" s="8" t="s">
         <v>832</v>
       </c>
@@ -11356,7 +11884,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="707" spans="2:3">
+    <row r="707" spans="1:3">
+      <c r="A707" t="s">
+        <v>5</v>
+      </c>
       <c r="B707" s="8" t="s">
         <v>833</v>
       </c>
@@ -11364,7 +11895,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="708" spans="2:3">
+    <row r="708" spans="1:3">
+      <c r="A708" t="s">
+        <v>5</v>
+      </c>
       <c r="B708" s="3" t="s">
         <v>834</v>
       </c>
@@ -11372,7 +11906,10 @@
         <v>44</v>
       </c>
     </row>
-    <row r="709" spans="2:3">
+    <row r="709" spans="1:3">
+      <c r="A709" t="s">
+        <v>5</v>
+      </c>
       <c r="B709" s="8" t="s">
         <v>835</v>
       </c>
@@ -11380,7 +11917,10 @@
         <v>36</v>
       </c>
     </row>
-    <row r="710" spans="2:3">
+    <row r="710" spans="1:3">
+      <c r="A710" t="s">
+        <v>5</v>
+      </c>
       <c r="B710" s="8" t="s">
         <v>836</v>
       </c>
@@ -11388,7 +11928,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="711" spans="2:3">
+    <row r="711" spans="1:3">
+      <c r="A711" t="s">
+        <v>5</v>
+      </c>
       <c r="B711" s="8" t="s">
         <v>837</v>
       </c>
@@ -11396,7 +11939,10 @@
         <v>32</v>
       </c>
     </row>
-    <row r="712" spans="2:3">
+    <row r="712" spans="1:3">
+      <c r="A712" t="s">
+        <v>5</v>
+      </c>
       <c r="B712" s="3" t="s">
         <v>838</v>
       </c>
@@ -11404,7 +11950,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="713" spans="2:3">
+    <row r="713" spans="1:3">
+      <c r="A713" t="s">
+        <v>5</v>
+      </c>
       <c r="B713" s="3" t="s">
         <v>839</v>
       </c>
@@ -11412,7 +11961,10 @@
         <v>36.5</v>
       </c>
     </row>
-    <row r="714" spans="2:3">
+    <row r="714" spans="1:3">
+      <c r="A714" t="s">
+        <v>5</v>
+      </c>
       <c r="B714" s="8" t="s">
         <v>840</v>
       </c>
@@ -11420,7 +11972,10 @@
         <v>56.5</v>
       </c>
     </row>
-    <row r="715" spans="2:3">
+    <row r="715" spans="1:3">
+      <c r="A715" t="s">
+        <v>5</v>
+      </c>
       <c r="B715" s="8" t="s">
         <v>841</v>
       </c>
@@ -11428,7 +11983,10 @@
         <v>35</v>
       </c>
     </row>
-    <row r="716" spans="2:3">
+    <row r="716" spans="1:3">
+      <c r="A716" t="s">
+        <v>5</v>
+      </c>
       <c r="B716" s="8" t="s">
         <v>842</v>
       </c>
@@ -11436,7 +11994,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="717" spans="2:3">
+    <row r="717" spans="1:3">
+      <c r="A717" t="s">
+        <v>5</v>
+      </c>
       <c r="B717" s="8" t="s">
         <v>843</v>
       </c>
@@ -11444,7 +12005,10 @@
         <v>31</v>
       </c>
     </row>
-    <row r="718" spans="2:3">
+    <row r="718" spans="1:3">
+      <c r="A718" t="s">
+        <v>5</v>
+      </c>
       <c r="B718" s="8" t="s">
         <v>844</v>
       </c>
@@ -11452,7 +12016,10 @@
         <v>40.5</v>
       </c>
     </row>
-    <row r="719" spans="2:3">
+    <row r="719" spans="1:3">
+      <c r="A719" t="s">
+        <v>5</v>
+      </c>
       <c r="B719" s="8" t="s">
         <v>845</v>
       </c>
@@ -11460,7 +12027,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="720" spans="2:3">
+    <row r="720" spans="1:3">
+      <c r="A720" t="s">
+        <v>5</v>
+      </c>
       <c r="B720" s="8" t="s">
         <v>846</v>
       </c>
@@ -11468,7 +12038,10 @@
         <v>125.8</v>
       </c>
     </row>
-    <row r="721" spans="2:3">
+    <row r="721" spans="1:3">
+      <c r="A721" t="s">
+        <v>5</v>
+      </c>
       <c r="B721" s="8" t="s">
         <v>847</v>
       </c>
@@ -11476,7 +12049,10 @@
         <v>125.8</v>
       </c>
     </row>
-    <row r="722" spans="2:3">
+    <row r="722" spans="1:3">
+      <c r="A722" t="s">
+        <v>5</v>
+      </c>
       <c r="B722" s="8" t="s">
         <v>848</v>
       </c>
@@ -11484,7 +12060,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="723" spans="2:3">
+    <row r="723" spans="1:3">
+      <c r="A723" t="s">
+        <v>5</v>
+      </c>
       <c r="B723" s="8" t="s">
         <v>849</v>
       </c>
@@ -11492,7 +12071,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="724" spans="2:3">
+    <row r="724" spans="1:3">
+      <c r="A724" t="s">
+        <v>5</v>
+      </c>
       <c r="B724" s="8" t="s">
         <v>850</v>
       </c>
@@ -11500,7 +12082,10 @@
         <v>126</v>
       </c>
     </row>
-    <row r="725" spans="2:3">
+    <row r="725" spans="1:3">
+      <c r="A725" t="s">
+        <v>5</v>
+      </c>
       <c r="B725" s="8" t="s">
         <v>851</v>
       </c>
@@ -11508,7 +12093,10 @@
         <v>97</v>
       </c>
     </row>
-    <row r="726" spans="2:3">
+    <row r="726" spans="1:3">
+      <c r="A726" t="s">
+        <v>5</v>
+      </c>
       <c r="B726" s="8" t="s">
         <v>852</v>
       </c>
@@ -11516,7 +12104,10 @@
         <v>88</v>
       </c>
     </row>
-    <row r="727" spans="2:3">
+    <row r="727" spans="1:3">
+      <c r="A727" t="s">
+        <v>5</v>
+      </c>
       <c r="B727" s="8" t="s">
         <v>853</v>
       </c>
@@ -11524,7 +12115,10 @@
         <v>71</v>
       </c>
     </row>
-    <row r="728" spans="2:3">
+    <row r="728" spans="1:3">
+      <c r="A728" t="s">
+        <v>5</v>
+      </c>
       <c r="B728" s="8" t="s">
         <v>854</v>
       </c>
@@ -11532,7 +12126,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="729" spans="2:3">
+    <row r="729" spans="1:3">
+      <c r="A729" t="s">
+        <v>5</v>
+      </c>
       <c r="B729" s="8" t="s">
         <v>855</v>
       </c>
@@ -11540,7 +12137,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="730" spans="2:3">
+    <row r="730" spans="1:3">
+      <c r="A730" t="s">
+        <v>5</v>
+      </c>
       <c r="B730" s="8" t="s">
         <v>856</v>
       </c>
@@ -11548,7 +12148,10 @@
         <v>41</v>
       </c>
     </row>
-    <row r="731" spans="2:3">
+    <row r="731" spans="1:3">
+      <c r="A731" t="s">
+        <v>5</v>
+      </c>
       <c r="B731" s="8" t="s">
         <v>857</v>
       </c>
@@ -11556,7 +12159,10 @@
         <v>41</v>
       </c>
     </row>
-    <row r="732" spans="2:3">
+    <row r="732" spans="1:3">
+      <c r="A732" t="s">
+        <v>5</v>
+      </c>
       <c r="B732" s="8" t="s">
         <v>858</v>
       </c>
@@ -11564,7 +12170,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="733" spans="2:3">
+    <row r="733" spans="1:3">
+      <c r="A733" t="s">
+        <v>5</v>
+      </c>
       <c r="B733" s="8" t="s">
         <v>859</v>
       </c>
@@ -11572,7 +12181,10 @@
         <v>54</v>
       </c>
     </row>
-    <row r="734" spans="2:3">
+    <row r="734" spans="1:3">
+      <c r="A734" t="s">
+        <v>5</v>
+      </c>
       <c r="B734" s="8" t="s">
         <v>860</v>
       </c>
@@ -11580,7 +12192,10 @@
         <v>78</v>
       </c>
     </row>
-    <row r="735" spans="2:3">
+    <row r="735" spans="1:3">
+      <c r="A735" t="s">
+        <v>5</v>
+      </c>
       <c r="B735" s="8" t="s">
         <v>861</v>
       </c>
@@ -11588,7 +12203,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="736" spans="2:3">
+    <row r="736" spans="1:3">
+      <c r="A736" t="s">
+        <v>5</v>
+      </c>
       <c r="B736" s="8" t="s">
         <v>862</v>
       </c>
@@ -11596,7 +12214,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="737" spans="2:3">
+    <row r="737" spans="1:3">
+      <c r="A737" t="s">
+        <v>5</v>
+      </c>
       <c r="B737" s="8" t="s">
         <v>863</v>
       </c>
@@ -11604,7 +12225,10 @@
         <v>96</v>
       </c>
     </row>
-    <row r="738" spans="2:3">
+    <row r="738" spans="1:3">
+      <c r="A738" t="s">
+        <v>5</v>
+      </c>
       <c r="B738" s="8" t="s">
         <v>864</v>
       </c>
@@ -11612,7 +12236,10 @@
         <v>96</v>
       </c>
     </row>
-    <row r="739" spans="2:3">
+    <row r="739" spans="1:3">
+      <c r="A739" t="s">
+        <v>5</v>
+      </c>
       <c r="B739" s="8" t="s">
         <v>865</v>
       </c>
@@ -11620,7 +12247,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="740" spans="2:3">
+    <row r="740" spans="1:3">
+      <c r="A740" t="s">
+        <v>5</v>
+      </c>
       <c r="B740" s="8" t="s">
         <v>866</v>
       </c>
@@ -11628,7 +12258,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="741" spans="2:3">
+    <row r="741" spans="1:3">
+      <c r="A741" t="s">
+        <v>5</v>
+      </c>
       <c r="B741" s="8" t="s">
         <v>867</v>
       </c>
@@ -11636,7 +12269,10 @@
         <v>91.8</v>
       </c>
     </row>
-    <row r="742" spans="2:3">
+    <row r="742" spans="1:3">
+      <c r="A742" t="s">
+        <v>5</v>
+      </c>
       <c r="B742" s="8" t="s">
         <v>868</v>
       </c>
@@ -11644,7 +12280,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="743" spans="2:3">
+    <row r="743" spans="1:3">
+      <c r="A743" t="s">
+        <v>5</v>
+      </c>
       <c r="B743" s="8" t="s">
         <v>869</v>
       </c>
@@ -11652,7 +12291,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="744" spans="2:3">
+    <row r="744" spans="1:3">
+      <c r="A744" t="s">
+        <v>5</v>
+      </c>
       <c r="B744" s="8" t="s">
         <v>870</v>
       </c>
@@ -11660,7 +12302,10 @@
         <v>116.6</v>
       </c>
     </row>
-    <row r="745" spans="2:3">
+    <row r="745" spans="1:3">
+      <c r="A745" t="s">
+        <v>5</v>
+      </c>
       <c r="B745" s="8" t="s">
         <v>871</v>
       </c>
@@ -11668,7 +12313,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="746" spans="2:3">
+    <row r="746" spans="1:3">
+      <c r="A746" t="s">
+        <v>5</v>
+      </c>
       <c r="B746" s="8" t="s">
         <v>872</v>
       </c>
@@ -11676,7 +12324,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="747" spans="2:3">
+    <row r="747" spans="1:3">
+      <c r="A747" t="s">
+        <v>5</v>
+      </c>
       <c r="B747" s="8" t="s">
         <v>873</v>
       </c>
@@ -11684,7 +12335,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="748" spans="2:3">
+    <row r="748" spans="1:3">
+      <c r="A748" t="s">
+        <v>5</v>
+      </c>
       <c r="B748" s="8" t="s">
         <v>874</v>
       </c>
@@ -11692,7 +12346,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="749" spans="2:3">
+    <row r="749" spans="1:3">
+      <c r="A749" t="s">
+        <v>5</v>
+      </c>
       <c r="B749" s="8" t="s">
         <v>875</v>
       </c>
@@ -11700,7 +12357,10 @@
         <v>90</v>
       </c>
     </row>
-    <row r="750" spans="2:3">
+    <row r="750" spans="1:3">
+      <c r="A750" t="s">
+        <v>5</v>
+      </c>
       <c r="B750" s="8" t="s">
         <v>876</v>
       </c>
@@ -11708,7 +12368,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="751" spans="2:3">
+    <row r="751" spans="1:3">
+      <c r="A751" t="s">
+        <v>5</v>
+      </c>
       <c r="B751" s="8" t="s">
         <v>877</v>
       </c>
@@ -11716,7 +12379,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="752" spans="2:3">
+    <row r="752" spans="1:3">
+      <c r="A752" t="s">
+        <v>5</v>
+      </c>
       <c r="B752" s="8" t="s">
         <v>878</v>
       </c>
@@ -11724,7 +12390,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="753" spans="2:3">
+    <row r="753" spans="1:3">
+      <c r="A753" t="s">
+        <v>5</v>
+      </c>
       <c r="B753" s="8" t="s">
         <v>879</v>
       </c>
@@ -11732,7 +12401,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="754" spans="2:3">
+    <row r="754" spans="1:3">
+      <c r="A754" t="s">
+        <v>5</v>
+      </c>
       <c r="B754" s="8" t="s">
         <v>880</v>
       </c>
@@ -11740,7 +12412,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="755" spans="2:3">
+    <row r="755" spans="1:3">
+      <c r="A755" t="s">
+        <v>5</v>
+      </c>
       <c r="B755" s="8" t="s">
         <v>881</v>
       </c>
@@ -11748,7 +12423,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="756" spans="2:3">
+    <row r="756" spans="1:3">
+      <c r="A756" t="s">
+        <v>5</v>
+      </c>
       <c r="B756" s="8" t="s">
         <v>882</v>
       </c>
@@ -11756,7 +12434,10 @@
         <v>69</v>
       </c>
     </row>
-    <row r="757" spans="2:3">
+    <row r="757" spans="1:3">
+      <c r="A757" t="s">
+        <v>5</v>
+      </c>
       <c r="B757" s="8" t="s">
         <v>883</v>
       </c>
@@ -11764,7 +12445,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="758" spans="2:3">
+    <row r="758" spans="1:3">
+      <c r="A758" t="s">
+        <v>5</v>
+      </c>
       <c r="B758" s="8" t="s">
         <v>884</v>
       </c>
@@ -11772,7 +12456,10 @@
         <v>92</v>
       </c>
     </row>
-    <row r="759" spans="2:3">
+    <row r="759" spans="1:3">
+      <c r="A759" t="s">
+        <v>5</v>
+      </c>
       <c r="B759" s="8" t="s">
         <v>885</v>
       </c>
@@ -11780,7 +12467,10 @@
         <v>29</v>
       </c>
     </row>
-    <row r="760" spans="2:3">
+    <row r="760" spans="1:3">
+      <c r="A760" t="s">
+        <v>5</v>
+      </c>
       <c r="B760" s="8" t="s">
         <v>886</v>
       </c>
@@ -11788,7 +12478,10 @@
         <v>29</v>
       </c>
     </row>
-    <row r="761" spans="2:3">
+    <row r="761" spans="1:3">
+      <c r="A761" t="s">
+        <v>5</v>
+      </c>
       <c r="B761" s="8" t="s">
         <v>887</v>
       </c>
@@ -11796,7 +12489,10 @@
         <v>75</v>
       </c>
     </row>
-    <row r="762" spans="2:3">
+    <row r="762" spans="1:3">
+      <c r="A762" t="s">
+        <v>5</v>
+      </c>
       <c r="B762" s="8" t="s">
         <v>888</v>
       </c>
@@ -11804,7 +12500,10 @@
         <v>75</v>
       </c>
     </row>
-    <row r="763" spans="2:3">
+    <row r="763" spans="1:3">
+      <c r="A763" t="s">
+        <v>5</v>
+      </c>
       <c r="B763" s="8" t="s">
         <v>889</v>
       </c>
@@ -11812,7 +12511,10 @@
         <v>106</v>
       </c>
     </row>
-    <row r="764" spans="2:3">
+    <row r="764" spans="1:3">
+      <c r="A764" t="s">
+        <v>5</v>
+      </c>
       <c r="B764" s="8" t="s">
         <v>890</v>
       </c>
@@ -11820,7 +12522,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="765" spans="2:3">
+    <row r="765" spans="1:3">
+      <c r="A765" t="s">
+        <v>5</v>
+      </c>
       <c r="B765" s="8" t="s">
         <v>891</v>
       </c>
@@ -11828,7 +12533,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="766" spans="2:3">
+    <row r="766" spans="1:3">
+      <c r="A766" t="s">
+        <v>5</v>
+      </c>
       <c r="B766" s="8" t="s">
         <v>892</v>
       </c>
@@ -11836,7 +12544,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="767" spans="2:3">
+    <row r="767" spans="1:3">
+      <c r="A767" t="s">
+        <v>5</v>
+      </c>
       <c r="B767" s="8" t="s">
         <v>893</v>
       </c>
@@ -11844,7 +12555,10 @@
         <v>63</v>
       </c>
     </row>
-    <row r="768" spans="2:3">
+    <row r="768" spans="1:3">
+      <c r="A768" t="s">
+        <v>5</v>
+      </c>
       <c r="B768" s="8" t="s">
         <v>894</v>
       </c>
@@ -11852,7 +12566,10 @@
         <v>63</v>
       </c>
     </row>
-    <row r="769" spans="2:3">
+    <row r="769" spans="1:3">
+      <c r="A769" t="s">
+        <v>5</v>
+      </c>
       <c r="B769" s="8" t="s">
         <v>895</v>
       </c>
@@ -11860,7 +12577,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="770" spans="2:3">
+    <row r="770" spans="1:3">
+      <c r="A770" t="s">
+        <v>5</v>
+      </c>
       <c r="B770" s="8" t="s">
         <v>896</v>
       </c>
@@ -11868,7 +12588,10 @@
         <v>54</v>
       </c>
     </row>
-    <row r="771" spans="2:3">
+    <row r="771" spans="1:3">
+      <c r="A771" t="s">
+        <v>5</v>
+      </c>
       <c r="B771" s="8" t="s">
         <v>897</v>
       </c>
@@ -11876,7 +12599,10 @@
         <v>33</v>
       </c>
     </row>
-    <row r="772" spans="2:3">
+    <row r="772" spans="1:3">
+      <c r="A772" t="s">
+        <v>5</v>
+      </c>
       <c r="B772" s="3" t="s">
         <v>898</v>
       </c>
@@ -11884,7 +12610,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="773" spans="2:3">
+    <row r="773" spans="1:3">
+      <c r="A773" t="s">
+        <v>5</v>
+      </c>
       <c r="B773" s="3" t="s">
         <v>899</v>
       </c>
@@ -11892,7 +12621,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="774" spans="2:3">
+    <row r="774" spans="1:3">
+      <c r="A774" t="s">
+        <v>5</v>
+      </c>
       <c r="B774" s="3" t="s">
         <v>900</v>
       </c>
@@ -11900,7 +12632,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="775" spans="2:3">
+    <row r="775" spans="1:3">
+      <c r="A775" t="s">
+        <v>5</v>
+      </c>
       <c r="B775" s="8" t="s">
         <v>901</v>
       </c>
@@ -11908,7 +12643,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="776" spans="2:3">
+    <row r="776" spans="1:3">
+      <c r="A776" t="s">
+        <v>5</v>
+      </c>
       <c r="B776" s="3" t="s">
         <v>902</v>
       </c>
@@ -11916,7 +12654,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="777" spans="2:3">
+    <row r="777" spans="1:3">
+      <c r="A777" t="s">
+        <v>5</v>
+      </c>
       <c r="B777" s="8" t="s">
         <v>903</v>
       </c>
@@ -11924,7 +12665,10 @@
         <v>65</v>
       </c>
     </row>
-    <row r="778" spans="2:3">
+    <row r="778" spans="1:3">
+      <c r="A778" t="s">
+        <v>5</v>
+      </c>
       <c r="B778" s="8" t="s">
         <v>904</v>
       </c>
@@ -11932,7 +12676,10 @@
         <v>64</v>
       </c>
     </row>
-    <row r="779" spans="2:3">
+    <row r="779" spans="1:3">
+      <c r="A779" t="s">
+        <v>5</v>
+      </c>
       <c r="B779" s="8" t="s">
         <v>905</v>
       </c>
@@ -11940,7 +12687,10 @@
         <v>64</v>
       </c>
     </row>
-    <row r="780" spans="2:3">
+    <row r="780" spans="1:3">
+      <c r="A780" t="s">
+        <v>5</v>
+      </c>
       <c r="B780" s="8" t="s">
         <v>906</v>
       </c>
@@ -11948,7 +12698,10 @@
         <v>33</v>
       </c>
     </row>
-    <row r="781" spans="2:3">
+    <row r="781" spans="1:3">
+      <c r="A781" t="s">
+        <v>5</v>
+      </c>
       <c r="B781" s="8" t="s">
         <v>907</v>
       </c>
@@ -11956,7 +12709,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="782" spans="2:3">
+    <row r="782" spans="1:3">
+      <c r="A782" t="s">
+        <v>5</v>
+      </c>
       <c r="B782" s="8" t="s">
         <v>908</v>
       </c>
@@ -11964,7 +12720,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="783" spans="2:3">
+    <row r="783" spans="1:3">
+      <c r="A783" t="s">
+        <v>5</v>
+      </c>
       <c r="B783" s="8" t="s">
         <v>909</v>
       </c>
@@ -11972,7 +12731,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="784" spans="2:3">
+    <row r="784" spans="1:3">
+      <c r="A784" t="s">
+        <v>5</v>
+      </c>
       <c r="B784" s="8" t="s">
         <v>910</v>
       </c>
@@ -11980,7 +12742,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="785" spans="2:3">
+    <row r="785" spans="1:3">
+      <c r="A785" t="s">
+        <v>5</v>
+      </c>
       <c r="B785" s="8" t="s">
         <v>911</v>
       </c>
@@ -11988,7 +12753,10 @@
         <v>54</v>
       </c>
     </row>
-    <row r="786" spans="2:3">
+    <row r="786" spans="1:3">
+      <c r="A786" t="s">
+        <v>5</v>
+      </c>
       <c r="B786" s="8" t="s">
         <v>912</v>
       </c>
@@ -11996,7 +12764,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="787" spans="2:3">
+    <row r="787" spans="1:3">
+      <c r="A787" t="s">
+        <v>5</v>
+      </c>
       <c r="B787" s="8" t="s">
         <v>913</v>
       </c>
@@ -12004,7 +12775,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="788" spans="2:3">
+    <row r="788" spans="1:3">
+      <c r="A788" t="s">
+        <v>5</v>
+      </c>
       <c r="B788" s="8" t="s">
         <v>914</v>
       </c>
@@ -12012,7 +12786,10 @@
         <v>88</v>
       </c>
     </row>
-    <row r="789" spans="2:3">
+    <row r="789" spans="1:3">
+      <c r="A789" t="s">
+        <v>5</v>
+      </c>
       <c r="B789" s="3" t="s">
         <v>915</v>
       </c>
@@ -12020,7 +12797,10 @@
         <v>109</v>
       </c>
     </row>
-    <row r="790" spans="2:3">
+    <row r="790" spans="1:3">
+      <c r="A790" t="s">
+        <v>5</v>
+      </c>
       <c r="B790" s="8" t="s">
         <v>916</v>
       </c>
@@ -12028,7 +12808,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="791" spans="2:3">
+    <row r="791" spans="1:3">
+      <c r="A791" t="s">
+        <v>5</v>
+      </c>
       <c r="B791" s="8" t="s">
         <v>917</v>
       </c>
@@ -12036,7 +12819,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="792" spans="2:3">
+    <row r="792" spans="1:3">
+      <c r="A792" t="s">
+        <v>5</v>
+      </c>
       <c r="B792" s="8" t="s">
         <v>918</v>
       </c>
@@ -12044,7 +12830,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="793" spans="2:3">
+    <row r="793" spans="1:3">
+      <c r="A793" t="s">
+        <v>5</v>
+      </c>
       <c r="B793" s="8" t="s">
         <v>919</v>
       </c>
@@ -12052,7 +12841,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="794" spans="2:3">
+    <row r="794" spans="1:3">
+      <c r="A794" t="s">
+        <v>5</v>
+      </c>
       <c r="B794" s="8" t="s">
         <v>920</v>
       </c>
@@ -12060,7 +12852,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="795" spans="2:3">
+    <row r="795" spans="1:3">
+      <c r="A795" t="s">
+        <v>5</v>
+      </c>
       <c r="B795" s="8" t="s">
         <v>921</v>
       </c>
@@ -12068,7 +12863,10 @@
         <v>405</v>
       </c>
     </row>
-    <row r="796" spans="2:3">
+    <row r="796" spans="1:3">
+      <c r="A796" t="s">
+        <v>5</v>
+      </c>
       <c r="B796" s="3" t="s">
         <v>922</v>
       </c>
@@ -12076,7 +12874,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="797" spans="2:3">
+    <row r="797" spans="1:3">
+      <c r="A797" t="s">
+        <v>5</v>
+      </c>
       <c r="B797" s="8" t="s">
         <v>923</v>
       </c>
@@ -12084,7 +12885,10 @@
         <v>53</v>
       </c>
     </row>
-    <row r="798" spans="2:3">
+    <row r="798" spans="1:3">
+      <c r="A798" t="s">
+        <v>5</v>
+      </c>
       <c r="B798" s="8" t="s">
         <v>924</v>
       </c>
@@ -12092,7 +12896,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="799" spans="2:3">
+    <row r="799" spans="1:3">
+      <c r="A799" t="s">
+        <v>5</v>
+      </c>
       <c r="B799" s="8" t="s">
         <v>925</v>
       </c>
@@ -12100,7 +12907,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="800" spans="2:3">
+    <row r="800" spans="1:3">
+      <c r="A800" t="s">
+        <v>5</v>
+      </c>
       <c r="B800" s="8" t="s">
         <v>926</v>
       </c>
@@ -12108,7 +12918,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="801" spans="2:3">
+    <row r="801" spans="1:3">
+      <c r="A801" t="s">
+        <v>5</v>
+      </c>
       <c r="B801" s="8" t="s">
         <v>927</v>
       </c>
@@ -12116,7 +12929,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="802" spans="2:3">
+    <row r="802" spans="1:3">
+      <c r="A802" t="s">
+        <v>5</v>
+      </c>
       <c r="B802" s="8" t="s">
         <v>928</v>
       </c>
@@ -12124,7 +12940,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="803" spans="2:3">
+    <row r="803" spans="1:3">
+      <c r="A803" t="s">
+        <v>5</v>
+      </c>
       <c r="B803" s="8" t="s">
         <v>929</v>
       </c>
@@ -12132,7 +12951,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="804" spans="2:3">
+    <row r="804" spans="1:3">
+      <c r="A804" t="s">
+        <v>5</v>
+      </c>
       <c r="B804" s="8" t="s">
         <v>930</v>
       </c>
@@ -12140,7 +12962,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="805" spans="2:3">
+    <row r="805" spans="1:3">
+      <c r="A805" t="s">
+        <v>5</v>
+      </c>
       <c r="B805" s="8" t="s">
         <v>931</v>
       </c>
@@ -12148,7 +12973,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="806" spans="2:3">
+    <row r="806" spans="1:3">
+      <c r="A806" t="s">
+        <v>5</v>
+      </c>
       <c r="B806" s="8" t="s">
         <v>932</v>
       </c>
@@ -12156,7 +12984,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="807" spans="2:3">
+    <row r="807" spans="1:3">
+      <c r="A807" t="s">
+        <v>5</v>
+      </c>
       <c r="B807" s="8" t="s">
         <v>933</v>
       </c>
@@ -12164,7 +12995,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="808" spans="2:3">
+    <row r="808" spans="1:3">
+      <c r="A808" t="s">
+        <v>5</v>
+      </c>
       <c r="B808" s="8" t="s">
         <v>934</v>
       </c>
@@ -12172,7 +13006,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="809" spans="2:3">
+    <row r="809" spans="1:3">
+      <c r="A809" t="s">
+        <v>5</v>
+      </c>
       <c r="B809" s="8" t="s">
         <v>935</v>
       </c>
@@ -12180,7 +13017,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="810" spans="2:3">
+    <row r="810" spans="1:3">
+      <c r="A810" t="s">
+        <v>5</v>
+      </c>
       <c r="B810" s="8" t="s">
         <v>936</v>
       </c>
@@ -12188,7 +13028,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="811" spans="2:3">
+    <row r="811" spans="1:3">
+      <c r="A811" t="s">
+        <v>5</v>
+      </c>
       <c r="B811" s="8" t="s">
         <v>937</v>
       </c>
@@ -12196,7 +13039,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="812" spans="2:3">
+    <row r="812" spans="1:3">
+      <c r="A812" t="s">
+        <v>5</v>
+      </c>
       <c r="B812" s="8" t="s">
         <v>938</v>
       </c>
@@ -12204,7 +13050,10 @@
         <v>74</v>
       </c>
     </row>
-    <row r="813" spans="2:3">
+    <row r="813" spans="1:3">
+      <c r="A813" t="s">
+        <v>5</v>
+      </c>
       <c r="B813" s="3" t="s">
         <v>939</v>
       </c>
@@ -12212,7 +13061,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="814" spans="2:3">
+    <row r="814" spans="1:3">
+      <c r="A814" t="s">
+        <v>5</v>
+      </c>
       <c r="B814" s="8" t="s">
         <v>940</v>
       </c>
@@ -12220,7 +13072,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="815" spans="2:3">
+    <row r="815" spans="1:3">
+      <c r="A815" t="s">
+        <v>5</v>
+      </c>
       <c r="B815" s="8" t="s">
         <v>941</v>
       </c>
@@ -12228,7 +13083,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="816" spans="2:3">
+    <row r="816" spans="1:3">
+      <c r="A816" t="s">
+        <v>5</v>
+      </c>
       <c r="B816" s="8" t="s">
         <v>942</v>
       </c>
@@ -12236,7 +13094,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="817" spans="2:3">
+    <row r="817" spans="1:3">
+      <c r="A817" t="s">
+        <v>5</v>
+      </c>
       <c r="B817" s="3" t="s">
         <v>943</v>
       </c>
@@ -12244,7 +13105,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="818" spans="2:3">
+    <row r="818" spans="1:3">
+      <c r="A818" t="s">
+        <v>5</v>
+      </c>
       <c r="B818" s="8" t="s">
         <v>944</v>
       </c>
@@ -12252,7 +13116,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="819" spans="2:3">
+    <row r="819" spans="1:3">
+      <c r="A819" t="s">
+        <v>5</v>
+      </c>
       <c r="B819" s="3" t="s">
         <v>945</v>
       </c>
@@ -12260,7 +13127,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="820" spans="2:3">
+    <row r="820" spans="1:3">
+      <c r="A820" t="s">
+        <v>5</v>
+      </c>
       <c r="B820" s="8" t="s">
         <v>946</v>
       </c>
@@ -12268,7 +13138,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="821" spans="2:3">
+    <row r="821" spans="1:3">
+      <c r="A821" t="s">
+        <v>5</v>
+      </c>
       <c r="B821" s="3" t="s">
         <v>947</v>
       </c>
@@ -12276,7 +13149,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="822" spans="2:3">
+    <row r="822" spans="1:3">
+      <c r="A822" t="s">
+        <v>5</v>
+      </c>
       <c r="B822" s="8" t="s">
         <v>948</v>
       </c>
@@ -12284,7 +13160,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="823" spans="2:3">
+    <row r="823" spans="1:3">
+      <c r="A823" t="s">
+        <v>5</v>
+      </c>
       <c r="B823" s="8" t="s">
         <v>949</v>
       </c>
@@ -12292,7 +13171,10 @@
         <v>46</v>
       </c>
     </row>
-    <row r="824" spans="2:3">
+    <row r="824" spans="1:3">
+      <c r="A824" t="s">
+        <v>5</v>
+      </c>
       <c r="B824" s="8" t="s">
         <v>950</v>
       </c>
@@ -12300,7 +13182,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="825" spans="2:3">
+    <row r="825" spans="1:3">
+      <c r="A825" t="s">
+        <v>5</v>
+      </c>
       <c r="B825" s="8" t="s">
         <v>951</v>
       </c>
@@ -12308,7 +13193,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="826" spans="2:3">
+    <row r="826" spans="1:3">
+      <c r="A826" t="s">
+        <v>5</v>
+      </c>
       <c r="B826" s="8" t="s">
         <v>952</v>
       </c>
@@ -12316,7 +13204,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="827" spans="2:3">
+    <row r="827" spans="1:3">
+      <c r="A827" t="s">
+        <v>5</v>
+      </c>
       <c r="B827" s="8" t="s">
         <v>953</v>
       </c>
@@ -12324,7 +13215,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="828" spans="2:3">
+    <row r="828" spans="1:3">
+      <c r="A828" t="s">
+        <v>5</v>
+      </c>
       <c r="B828" s="8" t="s">
         <v>954</v>
       </c>
@@ -12332,7 +13226,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="829" spans="2:3">
+    <row r="829" spans="1:3">
+      <c r="A829" t="s">
+        <v>5</v>
+      </c>
       <c r="B829" s="8" t="s">
         <v>955</v>
       </c>
@@ -12340,7 +13237,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="830" spans="2:3">
+    <row r="830" spans="1:3">
+      <c r="A830" t="s">
+        <v>5</v>
+      </c>
       <c r="B830" s="8" t="s">
         <v>956</v>
       </c>
@@ -12348,7 +13248,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="831" spans="2:3">
+    <row r="831" spans="1:3">
+      <c r="A831" t="s">
+        <v>5</v>
+      </c>
       <c r="B831" s="8" t="s">
         <v>957</v>
       </c>
@@ -12356,7 +13259,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="832" spans="2:3">
+    <row r="832" spans="1:3">
+      <c r="A832" t="s">
+        <v>5</v>
+      </c>
       <c r="B832" s="8" t="s">
         <v>958</v>
       </c>
@@ -12364,7 +13270,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="833" spans="2:3">
+    <row r="833" spans="1:3">
+      <c r="A833" t="s">
+        <v>5</v>
+      </c>
       <c r="B833" s="8" t="s">
         <v>959</v>
       </c>
@@ -12372,7 +13281,10 @@
         <v>665</v>
       </c>
     </row>
-    <row r="834" spans="2:3">
+    <row r="834" spans="1:3">
+      <c r="A834" t="s">
+        <v>5</v>
+      </c>
       <c r="B834" s="8" t="s">
         <v>960</v>
       </c>

</xml_diff>